<commit_message>
update for bleeding risk ECLS
</commit_message>
<xml_diff>
--- a/Analyses/Partner-Analyses-Metadata.xlsx
+++ b/Analyses/Partner-Analyses-Metadata.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioxfordnexus-my.sharepoint.com/personal/otss1968_ox_ac_uk/Documents/Documents/GitHub/CCP/Analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{356716B2-C3B1-498B-BBA3-AAA6A7893588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A09F8105-248B-4F6F-99B9-1D3D44B1EB6A}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{356716B2-C3B1-498B-BBA3-AAA6A7893588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{498FAF26-2B1B-41B8-99D6-0A73A05B2EAC}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Partner Analyses" sheetId="1" r:id="rId1"/>
     <sheet name="Sub-processors" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partner Analyses'!$A$3:$Z$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partner Analyses'!$A$3:$Z$59</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="326">
   <si>
     <t>ISARIC Partner Analyses</t>
   </si>
@@ -1194,6 +1194,20 @@
   <si>
     <t>Zainab KA Alaraji, Alnahrain University College of medicine, Iraq.</t>
   </si>
+  <si>
+    <t>Bleeding risk in ECLS</t>
+  </si>
+  <si>
+    <t>External validation of a bleeding risk prediction model in COVID-19 patients receiving extracorporeal life support using the ISARIC dataset</t>
+  </si>
+  <si>
+    <t>Externally validate a simplified bleeding-risk prediction model for patients receiving ECLS/ECMO using international datasets.
+Assess the model’s performance and generalizability across different healthcare settings.
+Support future research on risk-based monitoring and management during ECLS.</t>
+  </si>
+  <si>
+    <t>Daisuke Kasugai, MD, PhD ), Nagoya University Hospital, Japan</t>
+  </si>
 </sst>
 </file>
 
@@ -1207,11 +1221,18 @@
     <numFmt numFmtId="168" formatCode="ddmmmyyyy"/>
     <numFmt numFmtId="169" formatCode="dmmmyyyy"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1701,73 +1722,70 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1776,25 +1794,25 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1803,187 +1821,194 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2203,7 +2228,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1006"/>
+  <dimension ref="A1:Z1007"/>
   <sheetFormatPr defaultColWidth="14.46484375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="44.265625" customWidth="1"/>
@@ -2219,18 +2244,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
       <c r="K1" s="1"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
@@ -2249,16 +2274,16 @@
       <c r="Z1" s="2"/>
     </row>
     <row r="2" spans="1:26" ht="14.65" thickBot="1">
-      <c r="A2" s="84"/>
-      <c r="B2" s="84"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
+      <c r="A2" s="106"/>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="106"/>
+      <c r="I2" s="106"/>
+      <c r="J2" s="106"/>
       <c r="K2" s="1"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -2348,10 +2373,10 @@
       <c r="G4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="85" t="s">
+      <c r="H4" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="86"/>
+      <c r="I4" s="85"/>
       <c r="J4" s="14" t="s">
         <v>18</v>
       </c>
@@ -2394,10 +2419,10 @@
       <c r="G5" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="85" t="s">
+      <c r="H5" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="86"/>
+      <c r="I5" s="85"/>
       <c r="J5" s="14" t="s">
         <v>18</v>
       </c>
@@ -2471,10 +2496,10 @@
       <c r="Z6" s="9"/>
     </row>
     <row r="7" spans="1:26" ht="50.25" customHeight="1">
-      <c r="A7" s="92" t="s">
+      <c r="A7" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="87" t="s">
+      <c r="B7" s="98" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="58" t="s">
@@ -2489,13 +2514,13 @@
       <c r="F7" s="12">
         <v>44540</v>
       </c>
-      <c r="G7" s="90" t="s">
+      <c r="G7" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="91" t="s">
+      <c r="H7" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="91" t="s">
+      <c r="I7" s="89" t="s">
         <v>36</v>
       </c>
       <c r="J7" s="19" t="s">
@@ -2519,8 +2544,8 @@
       <c r="Z7" s="9"/>
     </row>
     <row r="8" spans="1:26" ht="30.75" customHeight="1">
-      <c r="A8" s="88"/>
-      <c r="B8" s="88"/>
+      <c r="A8" s="91"/>
+      <c r="B8" s="91"/>
       <c r="C8" s="58" t="s">
         <v>13</v>
       </c>
@@ -2533,9 +2558,9 @@
       <c r="F8" s="12">
         <v>44772</v>
       </c>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
+      <c r="G8" s="91"/>
+      <c r="H8" s="91"/>
+      <c r="I8" s="91"/>
       <c r="J8" s="19" t="s">
         <v>39</v>
       </c>
@@ -2557,8 +2582,8 @@
       <c r="Z8" s="9"/>
     </row>
     <row r="9" spans="1:26" ht="39.75" customHeight="1">
-      <c r="A9" s="88"/>
-      <c r="B9" s="88"/>
+      <c r="A9" s="91"/>
+      <c r="B9" s="91"/>
       <c r="C9" s="58" t="s">
         <v>13</v>
       </c>
@@ -2571,9 +2596,9 @@
       <c r="F9" s="12">
         <v>44817</v>
       </c>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
+      <c r="G9" s="91"/>
+      <c r="H9" s="91"/>
+      <c r="I9" s="91"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -2595,8 +2620,8 @@
       <c r="Z9" s="9"/>
     </row>
     <row r="10" spans="1:26" ht="47.25" customHeight="1">
-      <c r="A10" s="89"/>
-      <c r="B10" s="89"/>
+      <c r="A10" s="88"/>
+      <c r="B10" s="88"/>
       <c r="C10" s="58" t="s">
         <v>13</v>
       </c>
@@ -2609,9 +2634,9 @@
       <c r="F10" s="12">
         <v>45055</v>
       </c>
-      <c r="G10" s="89"/>
-      <c r="H10" s="89"/>
-      <c r="I10" s="89"/>
+      <c r="G10" s="88"/>
+      <c r="H10" s="88"/>
+      <c r="I10" s="88"/>
       <c r="J10" s="19" t="s">
         <v>39</v>
       </c>
@@ -2733,10 +2758,10 @@
       <c r="Z12" s="9"/>
     </row>
     <row r="13" spans="1:26" ht="66.75" customHeight="1">
-      <c r="A13" s="92" t="s">
+      <c r="A13" s="100" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="87" t="s">
+      <c r="B13" s="98" t="s">
         <v>56</v>
       </c>
       <c r="C13" s="60" t="s">
@@ -2751,16 +2776,16 @@
       <c r="F13" s="12">
         <v>44671</v>
       </c>
-      <c r="G13" s="90" t="s">
+      <c r="G13" s="86" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="90" t="s">
+      <c r="H13" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="I13" s="90" t="s">
+      <c r="I13" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="J13" s="91" t="s">
+      <c r="J13" s="89" t="s">
         <v>62</v>
       </c>
       <c r="K13" s="28">
@@ -2783,8 +2808,8 @@
       <c r="Z13" s="9"/>
     </row>
     <row r="14" spans="1:26" s="56" customFormat="1" ht="66.75" customHeight="1">
-      <c r="A14" s="93"/>
-      <c r="B14" s="94"/>
+      <c r="A14" s="101"/>
+      <c r="B14" s="102"/>
       <c r="C14" s="58" t="s">
         <v>13</v>
       </c>
@@ -2797,10 +2822,10 @@
       <c r="F14" s="12">
         <v>45072</v>
       </c>
-      <c r="G14" s="97"/>
-      <c r="H14" s="97"/>
-      <c r="I14" s="97"/>
-      <c r="J14" s="98"/>
+      <c r="G14" s="87"/>
+      <c r="H14" s="87"/>
+      <c r="I14" s="87"/>
+      <c r="J14" s="90"/>
       <c r="K14" s="28"/>
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
@@ -2819,8 +2844,8 @@
       <c r="Z14" s="9"/>
     </row>
     <row r="15" spans="1:26" ht="78.75" customHeight="1">
-      <c r="A15" s="89"/>
-      <c r="B15" s="89"/>
+      <c r="A15" s="88"/>
+      <c r="B15" s="88"/>
       <c r="C15" s="68" t="s">
         <v>13</v>
       </c>
@@ -2833,10 +2858,10 @@
       <c r="F15" s="71">
         <v>45981</v>
       </c>
-      <c r="G15" s="89"/>
-      <c r="H15" s="89"/>
-      <c r="I15" s="89"/>
-      <c r="J15" s="89"/>
+      <c r="G15" s="88"/>
+      <c r="H15" s="88"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
       <c r="K15" s="28"/>
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
@@ -2905,10 +2930,10 @@
       <c r="Z16" s="9"/>
     </row>
     <row r="17" spans="1:26" ht="45" customHeight="1">
-      <c r="A17" s="92" t="s">
+      <c r="A17" s="100" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="98" t="s">
         <v>71</v>
       </c>
       <c r="C17" s="58" t="s">
@@ -2923,7 +2948,7 @@
       <c r="F17" s="12">
         <v>44814</v>
       </c>
-      <c r="G17" s="90" t="s">
+      <c r="G17" s="86" t="s">
         <v>73</v>
       </c>
       <c r="H17" s="21" t="s">
@@ -2955,8 +2980,8 @@
       <c r="Z17" s="9"/>
     </row>
     <row r="18" spans="1:26" ht="102" customHeight="1">
-      <c r="A18" s="88"/>
-      <c r="B18" s="88"/>
+      <c r="A18" s="91"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="58" t="s">
         <v>13</v>
       </c>
@@ -2969,7 +2994,7 @@
       <c r="F18" s="12">
         <v>45331</v>
       </c>
-      <c r="G18" s="88"/>
+      <c r="G18" s="91"/>
       <c r="H18" s="21" t="s">
         <v>74</v>
       </c>
@@ -2997,8 +3022,8 @@
       <c r="Z18" s="9"/>
     </row>
     <row r="19" spans="1:26" ht="78" customHeight="1">
-      <c r="A19" s="88"/>
-      <c r="B19" s="89"/>
+      <c r="A19" s="91"/>
+      <c r="B19" s="88"/>
       <c r="C19" s="58" t="s">
         <v>13</v>
       </c>
@@ -3011,7 +3036,7 @@
       <c r="F19" s="12">
         <v>45266</v>
       </c>
-      <c r="G19" s="88"/>
+      <c r="G19" s="91"/>
       <c r="H19" s="21" t="s">
         <v>79</v>
       </c>
@@ -3233,10 +3258,10 @@
       <c r="Z23" s="9"/>
     </row>
     <row r="24" spans="1:26" ht="124.5" customHeight="1">
-      <c r="A24" s="95" t="s">
+      <c r="A24" s="103" t="s">
         <v>110</v>
       </c>
-      <c r="B24" s="87" t="s">
+      <c r="B24" s="98" t="s">
         <v>111</v>
       </c>
       <c r="C24" s="61" t="s">
@@ -3251,14 +3276,14 @@
       <c r="F24" s="12">
         <v>44809</v>
       </c>
-      <c r="G24" s="90" t="s">
+      <c r="G24" s="86" t="s">
         <v>114</v>
       </c>
-      <c r="H24" s="99" t="s">
+      <c r="H24" s="92" t="s">
         <v>115</v>
       </c>
-      <c r="I24" s="100"/>
-      <c r="J24" s="101"/>
+      <c r="I24" s="93"/>
+      <c r="J24" s="94"/>
       <c r="K24" s="15"/>
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
@@ -3277,8 +3302,8 @@
       <c r="Z24" s="9"/>
     </row>
     <row r="25" spans="1:26" ht="70.5" customHeight="1">
-      <c r="A25" s="89"/>
-      <c r="B25" s="89"/>
+      <c r="A25" s="88"/>
+      <c r="B25" s="88"/>
       <c r="C25" s="58" t="s">
         <v>13</v>
       </c>
@@ -3291,10 +3316,10 @@
       <c r="F25" s="12">
         <v>45534</v>
       </c>
-      <c r="G25" s="89"/>
-      <c r="H25" s="102"/>
-      <c r="I25" s="103"/>
-      <c r="J25" s="104"/>
+      <c r="G25" s="88"/>
+      <c r="H25" s="95"/>
+      <c r="I25" s="96"/>
+      <c r="J25" s="97"/>
       <c r="K25" s="15"/>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
@@ -3334,10 +3359,10 @@
       <c r="G26" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="H26" s="96" t="s">
+      <c r="H26" s="84" t="s">
         <v>122</v>
       </c>
-      <c r="I26" s="86"/>
+      <c r="I26" s="85"/>
       <c r="J26" s="14"/>
       <c r="K26" s="15" t="s">
         <v>30</v>
@@ -3359,10 +3384,10 @@
       <c r="Z26" s="9"/>
     </row>
     <row r="27" spans="1:26" ht="267" customHeight="1">
-      <c r="A27" s="92" t="s">
+      <c r="A27" s="100" t="s">
         <v>123</v>
       </c>
-      <c r="B27" s="87" t="s">
+      <c r="B27" s="98" t="s">
         <v>124</v>
       </c>
       <c r="C27" s="58" t="s">
@@ -3377,16 +3402,16 @@
       <c r="F27" s="12">
         <v>45190</v>
       </c>
-      <c r="G27" s="87" t="s">
+      <c r="G27" s="98" t="s">
         <v>126</v>
       </c>
-      <c r="H27" s="87" t="s">
+      <c r="H27" s="98" t="s">
         <v>127</v>
       </c>
-      <c r="I27" s="105" t="s">
+      <c r="I27" s="99" t="s">
         <v>128</v>
       </c>
-      <c r="J27" s="105" t="s">
+      <c r="J27" s="99" t="s">
         <v>127</v>
       </c>
       <c r="K27" s="35"/>
@@ -3407,8 +3432,8 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" spans="1:26" ht="42.75">
-      <c r="A28" s="89"/>
-      <c r="B28" s="89"/>
+      <c r="A28" s="88"/>
+      <c r="B28" s="88"/>
       <c r="C28" s="58" t="s">
         <v>13</v>
       </c>
@@ -3421,10 +3446,10 @@
       <c r="F28" s="12">
         <v>45400</v>
       </c>
-      <c r="G28" s="89"/>
-      <c r="H28" s="89"/>
-      <c r="I28" s="89"/>
-      <c r="J28" s="89"/>
+      <c r="G28" s="88"/>
+      <c r="H28" s="88"/>
+      <c r="I28" s="88"/>
+      <c r="J28" s="88"/>
       <c r="K28" s="15"/>
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
@@ -4484,25 +4509,25 @@
       <c r="Y52" s="9"/>
       <c r="Z52" s="9"/>
     </row>
-    <row r="53" spans="1:26" ht="57">
-      <c r="A53" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="B53" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="C53" s="58" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="45" t="s">
-        <v>226</v>
+    <row r="53" spans="1:26" s="82" customFormat="1" ht="84" customHeight="1">
+      <c r="A53" s="81" t="s">
+        <v>322</v>
+      </c>
+      <c r="B53" s="75" t="s">
+        <v>323</v>
+      </c>
+      <c r="C53" s="58"/>
+      <c r="D53" s="10" t="s">
+        <v>174</v>
       </c>
       <c r="E53" s="17"/>
       <c r="F53" s="12"/>
-      <c r="G53" s="13" t="s">
-        <v>269</v>
-      </c>
-      <c r="H53" s="13"/>
+      <c r="G53" s="109" t="s">
+        <v>324</v>
+      </c>
+      <c r="H53" s="80" t="s">
+        <v>325</v>
+      </c>
       <c r="I53" s="13"/>
       <c r="J53" s="13"/>
       <c r="K53" s="15"/>
@@ -4523,32 +4548,26 @@
       <c r="Z53" s="9"/>
     </row>
     <row r="54" spans="1:26" ht="57">
-      <c r="A54" s="18" t="s">
-        <v>270</v>
+      <c r="A54" s="13" t="s">
+        <v>267</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="C54" s="62"/>
+        <v>268</v>
+      </c>
+      <c r="C54" s="58" t="s">
+        <v>18</v>
+      </c>
       <c r="D54" s="45" t="s">
-        <v>272</v>
-      </c>
-      <c r="E54" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" s="46"/>
+        <v>226</v>
+      </c>
+      <c r="E54" s="17"/>
+      <c r="F54" s="12"/>
       <c r="G54" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="H54" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="I54" s="13" t="s">
-        <v>275</v>
-      </c>
-      <c r="J54" s="13" t="s">
-        <v>276</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="H54" s="13"/>
+      <c r="I54" s="13"/>
+      <c r="J54" s="13"/>
       <c r="K54" s="15"/>
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
@@ -4566,12 +4585,12 @@
       <c r="Y54" s="9"/>
       <c r="Z54" s="9"/>
     </row>
-    <row r="55" spans="1:26" ht="156.75">
-      <c r="A55" s="107" t="s">
-        <v>277</v>
+    <row r="55" spans="1:26" ht="57">
+      <c r="A55" s="18" t="s">
+        <v>270</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="C55" s="62"/>
       <c r="D55" s="45" t="s">
@@ -4582,16 +4601,16 @@
       </c>
       <c r="F55" s="46"/>
       <c r="G55" s="13" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="H55" s="13" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="I55" s="13" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="J55" s="13" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="K55" s="15"/>
       <c r="L55" s="9"/>
@@ -4610,12 +4629,12 @@
       <c r="Y55" s="9"/>
       <c r="Z55" s="9"/>
     </row>
-    <row r="56" spans="1:26" ht="71.25">
-      <c r="A56" s="18" t="s">
-        <v>283</v>
+    <row r="56" spans="1:26" ht="156.75">
+      <c r="A56" s="83" t="s">
+        <v>277</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C56" s="62"/>
       <c r="D56" s="45" t="s">
@@ -4626,20 +4645,18 @@
       </c>
       <c r="F56" s="46"/>
       <c r="G56" s="13" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="H56" s="13" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="I56" s="13" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="J56" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="K56" s="47">
-        <v>44213</v>
-      </c>
+        <v>282</v>
+      </c>
+      <c r="K56" s="15"/>
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9"/>
@@ -4656,12 +4673,12 @@
       <c r="Y56" s="9"/>
       <c r="Z56" s="9"/>
     </row>
-    <row r="57" spans="1:26" ht="96.75" customHeight="1">
+    <row r="57" spans="1:26" ht="71.25">
       <c r="A57" s="18" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C57" s="62"/>
       <c r="D57" s="45" t="s">
@@ -4672,18 +4689,20 @@
       </c>
       <c r="F57" s="46"/>
       <c r="G57" s="13" t="s">
-        <v>291</v>
-      </c>
-      <c r="H57" s="19" t="s">
-        <v>292</v>
+        <v>285</v>
+      </c>
+      <c r="H57" s="13" t="s">
+        <v>286</v>
       </c>
       <c r="I57" s="13" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="J57" s="13" t="s">
-        <v>294</v>
-      </c>
-      <c r="K57" s="15"/>
+        <v>288</v>
+      </c>
+      <c r="K57" s="47">
+        <v>44213</v>
+      </c>
       <c r="L57" s="9"/>
       <c r="M57" s="9"/>
       <c r="N57" s="9"/>
@@ -4700,32 +4719,34 @@
       <c r="Y57" s="9"/>
       <c r="Z57" s="9"/>
     </row>
-    <row r="58" spans="1:26" ht="180" customHeight="1">
-      <c r="A58" s="107" t="s">
-        <v>295</v>
+    <row r="58" spans="1:26" ht="96.75" customHeight="1">
+      <c r="A58" s="18" t="s">
+        <v>289</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="C58" s="62"/>
       <c r="D58" s="45" t="s">
         <v>272</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>297</v>
+        <v>13</v>
       </c>
       <c r="F58" s="46"/>
       <c r="G58" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="H58" s="96" t="s">
-        <v>299</v>
-      </c>
-      <c r="I58" s="86"/>
+        <v>291</v>
+      </c>
+      <c r="H58" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="I58" s="13" t="s">
+        <v>293</v>
+      </c>
       <c r="J58" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="K58" s="48"/>
+        <v>294</v>
+      </c>
+      <c r="K58" s="15"/>
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9"/>
@@ -4742,18 +4763,32 @@
       <c r="Y58" s="9"/>
       <c r="Z58" s="9"/>
     </row>
-    <row r="59" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A59" s="49"/>
-      <c r="B59" s="50"/>
-      <c r="C59" s="63"/>
-      <c r="D59" s="50"/>
-      <c r="E59" s="50"/>
-      <c r="F59" s="51"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="52"/>
-      <c r="K59" s="53"/>
+    <row r="59" spans="1:26" ht="180" customHeight="1">
+      <c r="A59" s="83" t="s">
+        <v>295</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="C59" s="62"/>
+      <c r="D59" s="45" t="s">
+        <v>272</v>
+      </c>
+      <c r="E59" s="45" t="s">
+        <v>297</v>
+      </c>
+      <c r="F59" s="46"/>
+      <c r="G59" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="H59" s="84" t="s">
+        <v>299</v>
+      </c>
+      <c r="I59" s="85"/>
+      <c r="J59" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="K59" s="48"/>
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9"/>
@@ -4771,7 +4806,7 @@
       <c r="Z59" s="9"/>
     </row>
     <row r="60" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A60" s="54"/>
+      <c r="A60" s="49"/>
       <c r="B60" s="50"/>
       <c r="C60" s="63"/>
       <c r="D60" s="50"/>
@@ -4860,7 +4895,7 @@
       <c r="C63" s="63"/>
       <c r="D63" s="50"/>
       <c r="E63" s="50"/>
-      <c r="F63" s="55"/>
+      <c r="F63" s="51"/>
       <c r="G63" s="52"/>
       <c r="H63" s="52"/>
       <c r="I63" s="52"/>
@@ -9447,7 +9482,7 @@
       <c r="Z226" s="9"/>
     </row>
     <row r="227" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A227" s="9"/>
+      <c r="A227" s="54"/>
       <c r="B227" s="50"/>
       <c r="C227" s="63"/>
       <c r="D227" s="50"/>
@@ -31286,9 +31321,53 @@
       <c r="Y1006" s="9"/>
       <c r="Z1006" s="9"/>
     </row>
+    <row r="1007" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A1007" s="9"/>
+      <c r="B1007" s="50"/>
+      <c r="C1007" s="63"/>
+      <c r="D1007" s="50"/>
+      <c r="E1007" s="50"/>
+      <c r="F1007" s="55"/>
+      <c r="G1007" s="52"/>
+      <c r="H1007" s="52"/>
+      <c r="I1007" s="52"/>
+      <c r="J1007" s="52"/>
+      <c r="K1007" s="53"/>
+      <c r="L1007" s="9"/>
+      <c r="M1007" s="9"/>
+      <c r="N1007" s="9"/>
+      <c r="O1007" s="9"/>
+      <c r="P1007" s="9"/>
+      <c r="Q1007" s="9"/>
+      <c r="R1007" s="9"/>
+      <c r="S1007" s="9"/>
+      <c r="T1007" s="9"/>
+      <c r="U1007" s="9"/>
+      <c r="V1007" s="9"/>
+      <c r="W1007" s="9"/>
+      <c r="X1007" s="9"/>
+      <c r="Y1007" s="9"/>
+      <c r="Z1007" s="9"/>
+    </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="G7:G10"/>
+    <mergeCell ref="H7:H10"/>
+    <mergeCell ref="I7:I10"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="H59:I59"/>
     <mergeCell ref="G13:G15"/>
     <mergeCell ref="H13:H15"/>
     <mergeCell ref="I13:I15"/>
@@ -31301,25 +31380,9 @@
     <mergeCell ref="H27:H28"/>
     <mergeCell ref="I27:I28"/>
     <mergeCell ref="J27:J28"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="G7:G10"/>
-    <mergeCell ref="H7:H10"/>
-    <mergeCell ref="I7:I10"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4:D58" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4:D59" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Published,Awaiting publication,Analysis underway,Analysis completed,On hold"</formula1>
     </dataValidation>
   </dataValidations>
@@ -31400,12 +31463,13 @@
     <hyperlink ref="C47" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
     <hyperlink ref="A48" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
     <hyperlink ref="A49" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="A54" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="A56" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="A57" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="A55" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="A57" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="A58" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
     <hyperlink ref="E37" r:id="rId80" xr:uid="{BE8A3D1F-7217-4106-97EB-5926D8F6809C}"/>
     <hyperlink ref="A51" r:id="rId81" xr:uid="{4C5DAD40-0EE6-4723-9972-DED6C1C412C8}"/>
     <hyperlink ref="A52" r:id="rId82" xr:uid="{AA4B0A3B-EFF0-43D2-8F6E-DAFE3F1EE47E}"/>
+    <hyperlink ref="A53" r:id="rId83" xr:uid="{F3A48EC8-A8EC-4902-BD1F-CB107258933F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -31424,13 +31488,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="108" t="s">
         <v>301</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
     </row>
     <row r="2" spans="1:5" ht="14.65" thickBot="1">
       <c r="A2" s="56"/>

</xml_diff>